<commit_message>
Updates for flights EOSS-394 and EOSS-395.  Also added a JSON-to-CSV conversion utility using 'jq'
</commit_message>
<xml_diff>
--- a/output/xlsx/flights_metadata.xlsx
+++ b/output/xlsx/flights_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="579">
   <si>
     <t>balloonsize</t>
   </si>
@@ -1727,6 +1727,30 @@
   </si>
   <si>
     <t>[{"altitude_ft":62992.0,"altitude_m":19199.96,"transition":"high_to_low"}]</t>
+  </si>
+  <si>
+    <t>2026-04-12</t>
+  </si>
+  <si>
+    <t>EOSS-394</t>
+  </si>
+  <si>
+    <t>2hrs 7mins 30secs</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":41952.0,"altitude_m":12786.97,"transition":"high_to_low"},{"altitude_ft":54733.0,"altitude_m":16682.62,"transition":"low_to_high"}]</t>
+  </si>
+  <si>
+    <t>["KC0D-2","K0SCC-13","AE0SS-4"]</t>
+  </si>
+  <si>
+    <t>EOSS-395</t>
+  </si>
+  <si>
+    <t>1hrs 55mins 29secs</t>
+  </si>
+  <si>
+    <t>[{"altitude_ft":12263.0,"altitude_m":3737.76,"transition":"low_to_high"},{"altitude_ft":64144.0,"altitude_m":19551.09,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -2058,7 +2082,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AT104"/>
+  <dimension ref="A1:AT106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:46">
@@ -16621,6 +16645,286 @@
         <v>1.75</v>
       </c>
     </row>
+    <row r="105" spans="1:46">
+      <c r="A105" t="s">
+        <v>62</v>
+      </c>
+      <c r="B105" t="s">
+        <v>566</v>
+      </c>
+      <c r="C105" t="s">
+        <v>571</v>
+      </c>
+      <c r="D105">
+        <v>91837</v>
+      </c>
+      <c r="E105">
+        <v>27991.92</v>
+      </c>
+      <c r="F105" t="b">
+        <v>1</v>
+      </c>
+      <c r="G105" t="s">
+        <v>572</v>
+      </c>
+      <c r="H105" t="s">
+        <v>573</v>
+      </c>
+      <c r="I105">
+        <v>7650</v>
+      </c>
+      <c r="J105" t="s">
+        <v>372</v>
+      </c>
+      <c r="K105">
+        <v>4595</v>
+      </c>
+      <c r="L105">
+        <v>1400.56</v>
+      </c>
+      <c r="M105">
+        <v>90.57</v>
+      </c>
+      <c r="N105">
+        <v>56.28</v>
+      </c>
+      <c r="O105">
+        <v>40.01166666666666</v>
+      </c>
+      <c r="P105">
+        <v>-103.12033333333332</v>
+      </c>
+      <c r="Q105">
+        <v>5216</v>
+      </c>
+      <c r="R105">
+        <v>1589.84</v>
+      </c>
+      <c r="S105">
+        <v>39.608</v>
+      </c>
+      <c r="T105">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U105" t="s">
+        <v>118</v>
+      </c>
+      <c r="V105">
+        <v>91612</v>
+      </c>
+      <c r="W105">
+        <v>27923.34</v>
+      </c>
+      <c r="X105">
+        <v>302</v>
+      </c>
+      <c r="Y105" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z105">
+        <v>12</v>
+      </c>
+      <c r="AA105">
+        <v>3.66</v>
+      </c>
+      <c r="AB105">
+        <v>0.79</v>
+      </c>
+      <c r="AC105">
+        <v>1.75</v>
+      </c>
+      <c r="AD105">
+        <v>90.57</v>
+      </c>
+      <c r="AE105">
+        <v>56.28</v>
+      </c>
+      <c r="AF105" t="s">
+        <v>574</v>
+      </c>
+      <c r="AG105">
+        <v>1.5</v>
+      </c>
+      <c r="AH105">
+        <v>3.31</v>
+      </c>
+      <c r="AI105">
+        <v>3.46</v>
+      </c>
+      <c r="AJ105">
+        <v>7.62</v>
+      </c>
+      <c r="AK105">
+        <v>1.65</v>
+      </c>
+      <c r="AL105">
+        <v>3.64</v>
+      </c>
+      <c r="AM105">
+        <v>7.4</v>
+      </c>
+      <c r="AN105">
+        <v>16.32</v>
+      </c>
+      <c r="AO105">
+        <v>8.12</v>
+      </c>
+      <c r="AP105">
+        <v>17.91</v>
+      </c>
+      <c r="AQ105">
+        <v>5.9</v>
+      </c>
+      <c r="AR105">
+        <v>13.01</v>
+      </c>
+      <c r="AS105">
+        <v>0.79</v>
+      </c>
+      <c r="AT105">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="106" spans="1:46">
+      <c r="A106" t="s">
+        <v>46</v>
+      </c>
+      <c r="B106" t="s">
+        <v>575</v>
+      </c>
+      <c r="C106" t="s">
+        <v>571</v>
+      </c>
+      <c r="D106">
+        <v>99167</v>
+      </c>
+      <c r="E106">
+        <v>30226.1</v>
+      </c>
+      <c r="F106" t="b">
+        <v>1</v>
+      </c>
+      <c r="G106" t="s">
+        <v>576</v>
+      </c>
+      <c r="H106" t="s">
+        <v>577</v>
+      </c>
+      <c r="I106">
+        <v>6929</v>
+      </c>
+      <c r="J106" t="s">
+        <v>263</v>
+      </c>
+      <c r="K106">
+        <v>4617</v>
+      </c>
+      <c r="L106">
+        <v>1407.26</v>
+      </c>
+      <c r="M106">
+        <v>85.13</v>
+      </c>
+      <c r="N106">
+        <v>52.9</v>
+      </c>
+      <c r="O106">
+        <v>39.89648333333333</v>
+      </c>
+      <c r="P106">
+        <v>-103.11896666666668</v>
+      </c>
+      <c r="Q106">
+        <v>5211</v>
+      </c>
+      <c r="R106">
+        <v>1588.31</v>
+      </c>
+      <c r="S106">
+        <v>39.608</v>
+      </c>
+      <c r="T106">
+        <v>-104.04216666666666</v>
+      </c>
+      <c r="U106" t="s">
+        <v>156</v>
+      </c>
+      <c r="V106">
+        <v>99059</v>
+      </c>
+      <c r="W106">
+        <v>30193.18</v>
+      </c>
+      <c r="X106">
+        <v>353</v>
+      </c>
+      <c r="Y106" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z106">
+        <v>12</v>
+      </c>
+      <c r="AA106">
+        <v>3.66</v>
+      </c>
+      <c r="AB106">
+        <v>0.77</v>
+      </c>
+      <c r="AC106">
+        <v>1.7</v>
+      </c>
+      <c r="AD106">
+        <v>85.13</v>
+      </c>
+      <c r="AE106">
+        <v>52.9</v>
+      </c>
+      <c r="AF106" t="s">
+        <v>578</v>
+      </c>
+      <c r="AG106">
+        <v>3</v>
+      </c>
+      <c r="AH106">
+        <v>6.61</v>
+      </c>
+      <c r="AI106">
+        <v>7.02</v>
+      </c>
+      <c r="AJ106">
+        <v>15.47</v>
+      </c>
+      <c r="AK106">
+        <v>2.08</v>
+      </c>
+      <c r="AL106">
+        <v>4.58</v>
+      </c>
+      <c r="AM106">
+        <v>12.86</v>
+      </c>
+      <c r="AN106">
+        <v>28.36</v>
+      </c>
+      <c r="AO106">
+        <v>12.44</v>
+      </c>
+      <c r="AP106">
+        <v>27.42</v>
+      </c>
+      <c r="AQ106">
+        <v>9.87</v>
+      </c>
+      <c r="AR106">
+        <v>21.75</v>
+      </c>
+      <c r="AS106">
+        <v>0.77</v>
+      </c>
+      <c r="AT106">
+        <v>1.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Corrected output data for EOSS-404
</commit_message>
<xml_diff>
--- a/output/xlsx/flights_metadata.xlsx
+++ b/output/xlsx/flights_metadata.xlsx
@@ -1870,13 +1870,13 @@
     <t>EOSS-404</t>
   </si>
   <si>
-    <t>5hrs 29mins 57secs</t>
+    <t>1hrs 17mins 30secs</t>
   </si>
   <si>
     <t>472</t>
   </si>
   <si>
-    <t>[{"altitude_ft":56551.0,"altitude_m":17236.74,"transition":"high_to_low"}]</t>
+    <t>[{"altitude_ft":56609.0,"altitude_m":17254.42,"transition":"high_to_low"}]</t>
   </si>
 </sst>
 </file>
@@ -18197,40 +18197,40 @@
         <v>618</v>
       </c>
       <c r="I115">
-        <v>19797.699</v>
+        <v>4650</v>
       </c>
       <c r="J115" t="s">
         <v>619</v>
       </c>
       <c r="K115">
-        <v>5590</v>
+        <v>6001</v>
       </c>
       <c r="L115">
-        <v>1703.83</v>
+        <v>1829.1</v>
       </c>
       <c r="M115">
-        <v>0.05</v>
+        <v>17.61</v>
       </c>
       <c r="N115">
-        <v>0.03</v>
+        <v>10.94</v>
       </c>
       <c r="O115">
-        <v>39.278</v>
+        <v>39.18613333333333</v>
       </c>
       <c r="P115">
-        <v>-103.496</v>
+        <v>-103.32883333333334</v>
       </c>
       <c r="Q115">
-        <v>5610</v>
+        <v>5606</v>
       </c>
       <c r="R115">
-        <v>1709.93</v>
+        <v>1708.71</v>
       </c>
       <c r="S115">
         <v>39.278166666666664</v>
       </c>
       <c r="T115">
-        <v>-103.4955</v>
+        <v>-103.49533333333332</v>
       </c>
       <c r="U115" t="s">
         <v>156</v>
@@ -18242,7 +18242,7 @@
         <v>20594.73</v>
       </c>
       <c r="X115">
-        <v>77</v>
+        <v>406</v>
       </c>
       <c r="Y115" t="s">
         <v>53</v>
@@ -18260,10 +18260,10 @@
         <v>1.7</v>
       </c>
       <c r="AD115">
-        <v>0.05</v>
+        <v>17.61</v>
       </c>
       <c r="AE115">
-        <v>0.03</v>
+        <v>10.94</v>
       </c>
       <c r="AF115" t="s">
         <v>620</v>

</xml_diff>